<commit_message>
update pkgs table intro
</commit_message>
<xml_diff>
--- a/packages.xlsx
+++ b/packages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/4216318/Desktop/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{168A1D6F-6A5B-D04B-AF69-9434BDE3C46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14115D1-30E8-C24C-AFCB-10D6C67F37E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2300" yWindow="-19920" windowWidth="34200" windowHeight="19660" activeTab="2" xr2:uid="{1A30A005-0681-6340-9241-9AE5FDFDA21E}"/>
   </bookViews>
@@ -106,15 +106,6 @@
     <t>$-$</t>
   </si>
   <si>
-    <t>\textbf{User utility}</t>
-  </si>
-  <si>
-    <t>\textbf{Imputed data} (\texttt{mids} object)</t>
-  </si>
-  <si>
-    <t>\textbf{Incomplete data} (\texttt{data.frame} object)</t>
-  </si>
-  <si>
     <t>$\pm$</t>
   </si>
   <si>
@@ -134,6 +125,15 @@
   </si>
   <si>
     <t>$-$ adaptability/publication readiness of visualizations</t>
+  </si>
+  <si>
+    <t>\textbf{Imputed data} (e.g., \texttt{mids} object)</t>
+  </si>
+  <si>
+    <t>\textbf{Incomplete data} (e.g., \texttt{data.frame} object)</t>
+  </si>
+  <si>
+    <t>\textbf{User utility}  (e.g., \texttt{ggplot} object)</t>
   </si>
 </sst>
 </file>
@@ -982,7 +982,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>18</v>
@@ -999,7 +999,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>20</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>20</v>
@@ -1025,7 +1025,7 @@
         <v>20</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>20</v>
@@ -1033,7 +1033,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>20</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>18</v>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>20</v>
@@ -1084,7 +1084,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>20</v>
@@ -1101,7 +1101,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>20</v>
@@ -1118,7 +1118,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>18</v>
@@ -1135,7 +1135,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>20</v>
@@ -1144,7 +1144,7 @@
         <v>21</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>21</v>
@@ -1152,7 +1152,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>20</v>

</xml_diff>